<commit_message>
Udemy Excel from beginning
</commit_message>
<xml_diff>
--- a/Udemy Excel 101.xlsx
+++ b/Udemy Excel 101.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8ef12d157d92b731/Documents/GitHub/Robert-Rookie-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8761CF19-0046-4715-B8FB-9230E793B6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{8761CF19-0046-4715-B8FB-9230E793B6F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42A629D9-F71F-4FF3-B08D-322117EDA3A6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9F602598-B120-46E6-997C-287E091787E5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>Monthly Budget</t>
   </si>
@@ -61,47 +61,14 @@
   <si>
     <t>Total</t>
   </si>
-  <si>
-    <t>Jan</t>
-  </si>
-  <si>
-    <t>Feb</t>
-  </si>
-  <si>
-    <t>Mar</t>
-  </si>
-  <si>
-    <t>April</t>
-  </si>
-  <si>
-    <t>May</t>
-  </si>
-  <si>
-    <t>Jun</t>
-  </si>
-  <si>
-    <t>July</t>
-  </si>
-  <si>
-    <t>Aug</t>
-  </si>
-  <si>
-    <t>Sept</t>
-  </si>
-  <si>
-    <t>Oct</t>
-  </si>
-  <si>
-    <t>Nov</t>
-  </si>
-  <si>
-    <t>Dec</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="mmm\-yyyy"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -131,8 +98,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,6 +439,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" customWidth="1"/>
+    <col min="2" max="13" width="12.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -482,41 +451,41 @@
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" t="s">
-        <v>17</v>
-      </c>
-      <c r="L3" t="s">
-        <v>18</v>
-      </c>
-      <c r="M3" t="s">
-        <v>19</v>
+      <c r="B3" s="1">
+        <v>45658</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45689</v>
+      </c>
+      <c r="D3" s="1">
+        <v>45717</v>
+      </c>
+      <c r="E3" s="1">
+        <v>45748</v>
+      </c>
+      <c r="F3" s="1">
+        <v>45778</v>
+      </c>
+      <c r="G3" s="1">
+        <v>45809</v>
+      </c>
+      <c r="H3" s="1">
+        <v>45839</v>
+      </c>
+      <c r="I3" s="1">
+        <v>45870</v>
+      </c>
+      <c r="J3" s="1">
+        <v>45901</v>
+      </c>
+      <c r="K3" s="1">
+        <v>45931</v>
+      </c>
+      <c r="L3" s="1">
+        <v>45962</v>
+      </c>
+      <c r="M3" s="1">
+        <v>45992</v>
       </c>
       <c r="N3" t="s">
         <v>7</v>

</xml_diff>